<commit_message>
update templates to latest
</commit_message>
<xml_diff>
--- a/templates/ERC000011/metadata_template_ERC000011.xlsx
+++ b/templates/ERC000011/metadata_template_ERC000011.xlsx
@@ -17,14 +17,14 @@
     <sheet name="cv_sample" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="environmentalsample">'cv_sample'!$P$1:$P$2</definedName>
+    <definedName name="environmentalsample">'cv_sample'!$Q$1:$Q$2</definedName>
     <definedName name="fileformat">'cv_run'!$D$1:$D$24</definedName>
-    <definedName name="geographiclocationcountryandorsea">'cv_sample'!$S$1:$S$289</definedName>
-    <definedName name="instrumentmodel">'cv_experiment'!$N$1:$N$87</definedName>
+    <definedName name="geographiclocationcountryandorsea">'cv_sample'!$T$1:$T$294</definedName>
+    <definedName name="instrumentmodel">'cv_experiment'!$N$1:$N$88</definedName>
     <definedName name="libraryselection">'cv_experiment'!$I$1:$I$31</definedName>
     <definedName name="librarysource">'cv_experiment'!$H$1:$H$9</definedName>
     <definedName name="librarystrategy">'cv_experiment'!$G$1:$G$41</definedName>
-    <definedName name="platform">'cv_experiment'!$M$1:$M$17</definedName>
+    <definedName name="platform">'cv_experiment'!$M$1:$M$18</definedName>
     <definedName name="studytype">'cv_study'!$C$1:$C$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="630">
   <si>
     <t>alias</t>
   </si>
@@ -448,6 +448,9 @@
     <t>ELEMENT</t>
   </si>
   <si>
+    <t>AVITI</t>
+  </si>
+  <si>
     <t>ULTIMA</t>
   </si>
   <si>
@@ -538,6 +541,9 @@
     <t>AB SOLiD System 3.0</t>
   </si>
   <si>
+    <t>AVITI 24</t>
+  </si>
+  <si>
     <t>BGISEQ-50</t>
   </si>
   <si>
@@ -838,6 +844,12 @@
     <t>(Mandatory) Ncbi taxonomy identifier.  this is appropriate for individual organisms and some environmental samples.</t>
   </si>
   <si>
+    <t>scientific_name</t>
+  </si>
+  <si>
+    <t>(Optional) Scientific name of sample that distinguishes its taxonomy.  please use a name or synonym that is tracked in the insdc taxonomy database. also, this field can be used to confirm the taxon_id setting.</t>
+  </si>
+  <si>
     <t>sample_description</t>
   </si>
   <si>
@@ -1147,9 +1159,6 @@
     <t>Dominican Republic</t>
   </si>
   <si>
-    <t>East Timor</t>
-  </si>
-  <si>
     <t>Ecuador</t>
   </si>
   <si>
@@ -1168,6 +1177,9 @@
     <t>Estonia</t>
   </si>
   <si>
+    <t>Eswatini</t>
+  </si>
+  <si>
     <t>Ethiopia</t>
   </si>
   <si>
@@ -1369,6 +1381,9 @@
     <t>Liechtenstein</t>
   </si>
   <si>
+    <t>Line Islands</t>
+  </si>
+  <si>
     <t>Lithuania</t>
   </si>
   <si>
@@ -1378,9 +1393,6 @@
     <t>Macau</t>
   </si>
   <si>
-    <t>Macedonia</t>
-  </si>
-  <si>
     <t>Madagascar</t>
   </si>
   <si>
@@ -1420,7 +1432,7 @@
     <t>Mexico</t>
   </si>
   <si>
-    <t>Micronesia</t>
+    <t>Micronesia, Federated States of</t>
   </si>
   <si>
     <t>Midway Islands</t>
@@ -1489,6 +1501,9 @@
     <t>North Korea</t>
   </si>
   <si>
+    <t>North Macedonia</t>
+  </si>
+  <si>
     <t>North Sea</t>
   </si>
   <si>
@@ -1564,6 +1579,9 @@
     <t>Rwanda</t>
   </si>
   <si>
+    <t>Saint Barthelemy</t>
+  </si>
+  <si>
     <t>Saint Helena</t>
   </si>
   <si>
@@ -1585,6 +1603,9 @@
     <t>San Marino</t>
   </si>
   <si>
+    <t>Saint Martin</t>
+  </si>
+  <si>
     <t>Sao Tome and Principe</t>
   </si>
   <si>
@@ -1630,6 +1651,9 @@
     <t>South Korea</t>
   </si>
   <si>
+    <t>South Sudan</t>
+  </si>
+  <si>
     <t>Southern Ocean</t>
   </si>
   <si>
@@ -1642,6 +1666,9 @@
     <t>Sri Lanka</t>
   </si>
   <si>
+    <t>State of Palestine</t>
+  </si>
+  <si>
     <t>Sudan</t>
   </si>
   <si>
@@ -1651,9 +1678,6 @@
     <t>Svalbard</t>
   </si>
   <si>
-    <t>Swaziland</t>
-  </si>
-  <si>
     <t>Sweden</t>
   </si>
   <si>
@@ -1678,6 +1702,9 @@
     <t>Thailand</t>
   </si>
   <si>
+    <t>Timor-Leste</t>
+  </si>
+  <si>
     <t>Togo</t>
   </si>
   <si>
@@ -1738,10 +1765,10 @@
     <t>Viet Nam</t>
   </si>
   <si>
+    <t>Wake Island</t>
+  </si>
+  <si>
     <t>Virgin Islands</t>
-  </si>
-  <si>
-    <t>Wake Island</t>
   </si>
   <si>
     <t>Wallis and Futuna</t>
@@ -2421,10 +2448,10 @@
         <v>124</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="150" customHeight="1">
@@ -2465,10 +2492,10 @@
         <v>125</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -2495,7 +2522,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="G1:N87"/>
+  <dimension ref="G1:N88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="7:14">
@@ -2512,7 +2539,7 @@
         <v>126</v>
       </c>
       <c r="N1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" spans="7:14">
@@ -2529,7 +2556,7 @@
         <v>127</v>
       </c>
       <c r="N2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3" spans="7:14">
@@ -2546,7 +2573,7 @@
         <v>128</v>
       </c>
       <c r="N3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="7:14">
@@ -2563,7 +2590,7 @@
         <v>129</v>
       </c>
       <c r="N4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="7:14">
@@ -2580,7 +2607,7 @@
         <v>130</v>
       </c>
       <c r="N5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="7:14">
@@ -2597,7 +2624,7 @@
         <v>131</v>
       </c>
       <c r="N6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" spans="7:14">
@@ -2614,7 +2641,7 @@
         <v>132</v>
       </c>
       <c r="N7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8" spans="7:14">
@@ -2631,7 +2658,7 @@
         <v>133</v>
       </c>
       <c r="N8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="7:14">
@@ -2648,7 +2675,7 @@
         <v>134</v>
       </c>
       <c r="N9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="7:14">
@@ -2662,7 +2689,7 @@
         <v>135</v>
       </c>
       <c r="N10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="7:14">
@@ -2676,7 +2703,7 @@
         <v>136</v>
       </c>
       <c r="N11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="7:14">
@@ -2690,7 +2717,7 @@
         <v>137</v>
       </c>
       <c r="N12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="7:14">
@@ -2704,7 +2731,7 @@
         <v>138</v>
       </c>
       <c r="N13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="7:14">
@@ -2718,7 +2745,7 @@
         <v>139</v>
       </c>
       <c r="N14" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="7:14">
@@ -2732,7 +2759,7 @@
         <v>140</v>
       </c>
       <c r="N15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="7:14">
@@ -2746,7 +2773,7 @@
         <v>141</v>
       </c>
       <c r="N16" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="7:14">
@@ -2760,7 +2787,7 @@
         <v>142</v>
       </c>
       <c r="N17" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="7:14">
@@ -2770,8 +2797,11 @@
       <c r="I18" t="s">
         <v>54</v>
       </c>
+      <c r="M18" t="s">
+        <v>143</v>
+      </c>
       <c r="N18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="7:14">
@@ -2782,7 +2812,7 @@
         <v>105</v>
       </c>
       <c r="N19" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="7:14">
@@ -2793,7 +2823,7 @@
         <v>106</v>
       </c>
       <c r="N20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="7:14">
@@ -2804,7 +2834,7 @@
         <v>107</v>
       </c>
       <c r="N21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" spans="7:14">
@@ -2815,7 +2845,7 @@
         <v>108</v>
       </c>
       <c r="N22" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="23" spans="7:14">
@@ -2826,7 +2856,7 @@
         <v>109</v>
       </c>
       <c r="N23" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="24" spans="7:14">
@@ -2837,7 +2867,7 @@
         <v>110</v>
       </c>
       <c r="N24" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25" spans="7:14">
@@ -2848,7 +2878,7 @@
         <v>111</v>
       </c>
       <c r="N25" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="7:14">
@@ -2859,7 +2889,7 @@
         <v>112</v>
       </c>
       <c r="N26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="27" spans="7:14">
@@ -2870,7 +2900,7 @@
         <v>113</v>
       </c>
       <c r="N27" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="28" spans="7:14">
@@ -2881,7 +2911,7 @@
         <v>114</v>
       </c>
       <c r="N28" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="29" spans="7:14">
@@ -2892,7 +2922,7 @@
         <v>115</v>
       </c>
       <c r="N29" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30" spans="7:14">
@@ -2903,7 +2933,7 @@
         <v>116</v>
       </c>
       <c r="N30" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" spans="7:14">
@@ -2914,7 +2944,7 @@
         <v>117</v>
       </c>
       <c r="N31" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="7:14">
@@ -2922,7 +2952,7 @@
         <v>66</v>
       </c>
       <c r="N32" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="33" spans="7:14">
@@ -2930,7 +2960,7 @@
         <v>67</v>
       </c>
       <c r="N33" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" spans="7:14">
@@ -2938,7 +2968,7 @@
         <v>68</v>
       </c>
       <c r="N34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="35" spans="7:14">
@@ -2946,7 +2976,7 @@
         <v>69</v>
       </c>
       <c r="N35" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" spans="7:14">
@@ -2954,7 +2984,7 @@
         <v>70</v>
       </c>
       <c r="N36" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="37" spans="7:14">
@@ -2962,7 +2992,7 @@
         <v>71</v>
       </c>
       <c r="N37" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="38" spans="7:14">
@@ -2970,7 +3000,7 @@
         <v>72</v>
       </c>
       <c r="N38" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="39" spans="7:14">
@@ -2978,7 +3008,7 @@
         <v>73</v>
       </c>
       <c r="N39" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="40" spans="7:14">
@@ -2986,7 +3016,7 @@
         <v>74</v>
       </c>
       <c r="N40" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="41" spans="7:14">
@@ -2994,236 +3024,241 @@
         <v>75</v>
       </c>
       <c r="N41" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="42" spans="7:14">
       <c r="N42" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="43" spans="7:14">
       <c r="N43" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="44" spans="7:14">
       <c r="N44" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="45" spans="7:14">
       <c r="N45" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="46" spans="7:14">
       <c r="N46" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="47" spans="7:14">
       <c r="N47" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="48" spans="7:14">
       <c r="N48" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="49" spans="14:14">
       <c r="N49" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50" spans="14:14">
       <c r="N50" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="51" spans="14:14">
       <c r="N51" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="52" spans="14:14">
       <c r="N52" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="53" spans="14:14">
       <c r="N53" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="54" spans="14:14">
       <c r="N54" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="55" spans="14:14">
       <c r="N55" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="56" spans="14:14">
       <c r="N56" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="57" spans="14:14">
       <c r="N57" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="58" spans="14:14">
       <c r="N58" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="59" spans="14:14">
       <c r="N59" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="60" spans="14:14">
       <c r="N60" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="61" spans="14:14">
       <c r="N61" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="62" spans="14:14">
       <c r="N62" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="63" spans="14:14">
       <c r="N63" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="64" spans="14:14">
       <c r="N64" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="65" spans="14:14">
       <c r="N65" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="66" spans="14:14">
       <c r="N66" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="67" spans="14:14">
       <c r="N67" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="68" spans="14:14">
       <c r="N68" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="69" spans="14:14">
       <c r="N69" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="70" spans="14:14">
       <c r="N70" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="71" spans="14:14">
       <c r="N71" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="72" spans="14:14">
       <c r="N72" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="73" spans="14:14">
       <c r="N73" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="74" spans="14:14">
       <c r="N74" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="75" spans="14:14">
       <c r="N75" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="76" spans="14:14">
       <c r="N76" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="77" spans="14:14">
       <c r="N77" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="78" spans="14:14">
       <c r="N78" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="79" spans="14:14">
       <c r="N79" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="80" spans="14:14">
       <c r="N80" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="81" spans="14:14">
       <c r="N81" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="82" spans="14:14">
       <c r="N82" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="83" spans="14:14">
       <c r="N83" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="84" spans="14:14">
       <c r="N84" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="85" spans="14:14">
       <c r="N85" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="86" spans="14:14">
       <c r="N86" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="87" spans="14:14">
       <c r="N87" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="88" spans="14:14">
+      <c r="N88" t="s">
         <v>117</v>
       </c>
     </row>
@@ -3245,27 +3280,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="150" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -3285,122 +3320,122 @@
   <sheetData>
     <row r="1" spans="4:4">
       <c r="D1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="4:4">
       <c r="D2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="4:4">
       <c r="D3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="4" spans="4:4">
       <c r="D4" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="5" spans="4:4">
       <c r="D5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" spans="4:4">
       <c r="D6" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="4:4">
       <c r="D7" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="4:4">
       <c r="D8" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" spans="4:4">
       <c r="D9" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="4:4">
       <c r="D10" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="4:4">
       <c r="D12" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="13" spans="4:4">
       <c r="D13" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="14" spans="4:4">
       <c r="D14" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="4:4">
       <c r="D15" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" spans="4:4">
       <c r="D16" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" spans="4:4">
       <c r="D17" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" spans="4:4">
       <c r="D18" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="19" spans="4:4">
       <c r="D19" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="20" spans="4:4">
       <c r="D20" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="21" spans="4:4">
       <c r="D21" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="22" spans="4:4">
       <c r="D22" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="4:4">
       <c r="D23" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="24" spans="4:4">
       <c r="D24" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -3410,13 +3445,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="301" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34">
+    <row r="1" spans="1:35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3424,212 +3459,218 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>294</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>589</v>
+        <v>302</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>593</v>
+        <v>600</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>595</v>
+        <v>602</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>599</v>
+        <v>606</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>603</v>
+        <v>610</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>605</v>
+        <v>612</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>607</v>
+        <v>614</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>609</v>
+        <v>616</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>611</v>
+        <v>618</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>613</v>
+        <v>620</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>615</v>
+        <v>622</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>617</v>
+        <v>624</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="2" spans="1:34" ht="150" customHeight="1">
+        <v>626</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" ht="150" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>295</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>590</v>
+        <v>303</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>596</v>
+        <v>603</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>598</v>
+        <v>605</v>
       </c>
       <c r="X2" s="2" t="s">
-        <v>600</v>
+        <v>607</v>
       </c>
       <c r="Y2" s="2" t="s">
-        <v>602</v>
+        <v>609</v>
       </c>
       <c r="Z2" s="2" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
       <c r="AA2" s="2" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
       <c r="AB2" s="2" t="s">
-        <v>608</v>
+        <v>615</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="AD2" s="2" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>614</v>
+        <v>621</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>616</v>
+        <v>623</v>
       </c>
       <c r="AG2" s="2" t="s">
-        <v>618</v>
+        <v>625</v>
       </c>
       <c r="AH2" s="2" t="s">
-        <v>620</v>
+        <v>627</v>
+      </c>
+      <c r="AI2" s="2" t="s">
+        <v>629</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:P101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q3:Q101">
       <formula1>environmentalsample</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S3:S101">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T3:T101">
       <formula1>geographiclocationcountryandorsea</formula1>
     </dataValidation>
   </dataValidations>
@@ -3639,1458 +3680,1483 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="P1:S289"/>
+  <dimension ref="Q1:T294"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="16:19">
-      <c r="P1" t="s">
-        <v>292</v>
-      </c>
-      <c r="S1" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="2" spans="16:19">
-      <c r="P2" t="s">
-        <v>293</v>
-      </c>
-      <c r="S2" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="3" spans="16:19">
-      <c r="S3" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="4" spans="16:19">
-      <c r="S4" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="5" spans="16:19">
-      <c r="S5" t="s">
+    <row r="1" spans="17:20">
+      <c r="Q1" t="s">
+        <v>296</v>
+      </c>
+      <c r="T1" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="6" spans="16:19">
-      <c r="S6" t="s">
+    <row r="2" spans="17:20">
+      <c r="Q2" t="s">
+        <v>297</v>
+      </c>
+      <c r="T2" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="7" spans="16:19">
-      <c r="S7" t="s">
+    <row r="3" spans="17:20">
+      <c r="T3" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="8" spans="16:19">
-      <c r="S8" t="s">
+    <row r="4" spans="17:20">
+      <c r="T4" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="9" spans="16:19">
-      <c r="S9" t="s">
+    <row r="5" spans="17:20">
+      <c r="T5" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="10" spans="16:19">
-      <c r="S10" t="s">
+    <row r="6" spans="17:20">
+      <c r="T6" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="11" spans="16:19">
-      <c r="S11" t="s">
+    <row r="7" spans="17:20">
+      <c r="T7" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="12" spans="16:19">
-      <c r="S12" t="s">
+    <row r="8" spans="17:20">
+      <c r="T8" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="13" spans="16:19">
-      <c r="S13" t="s">
+    <row r="9" spans="17:20">
+      <c r="T9" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="14" spans="16:19">
-      <c r="S14" t="s">
+    <row r="10" spans="17:20">
+      <c r="T10" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="15" spans="16:19">
-      <c r="S15" t="s">
+    <row r="11" spans="17:20">
+      <c r="T11" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="16" spans="16:19">
-      <c r="S16" t="s">
+    <row r="12" spans="17:20">
+      <c r="T12" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="17" spans="19:19">
-      <c r="S17" t="s">
+    <row r="13" spans="17:20">
+      <c r="T13" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="18" spans="19:19">
-      <c r="S18" t="s">
+    <row r="14" spans="17:20">
+      <c r="T14" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="19" spans="19:19">
-      <c r="S19" t="s">
+    <row r="15" spans="17:20">
+      <c r="T15" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="20" spans="19:19">
-      <c r="S20" t="s">
+    <row r="16" spans="17:20">
+      <c r="T16" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="21" spans="19:19">
-      <c r="S21" t="s">
+    <row r="17" spans="20:20">
+      <c r="T17" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="22" spans="19:19">
-      <c r="S22" t="s">
+    <row r="18" spans="20:20">
+      <c r="T18" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="23" spans="19:19">
-      <c r="S23" t="s">
+    <row r="19" spans="20:20">
+      <c r="T19" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="24" spans="19:19">
-      <c r="S24" t="s">
+    <row r="20" spans="20:20">
+      <c r="T20" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="25" spans="19:19">
-      <c r="S25" t="s">
+    <row r="21" spans="20:20">
+      <c r="T21" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="26" spans="19:19">
-      <c r="S26" t="s">
+    <row r="22" spans="20:20">
+      <c r="T22" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="27" spans="19:19">
-      <c r="S27" t="s">
+    <row r="23" spans="20:20">
+      <c r="T23" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="28" spans="19:19">
-      <c r="S28" t="s">
+    <row r="24" spans="20:20">
+      <c r="T24" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="29" spans="19:19">
-      <c r="S29" t="s">
+    <row r="25" spans="20:20">
+      <c r="T25" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="30" spans="19:19">
-      <c r="S30" t="s">
+    <row r="26" spans="20:20">
+      <c r="T26" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="31" spans="19:19">
-      <c r="S31" t="s">
+    <row r="27" spans="20:20">
+      <c r="T27" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="32" spans="19:19">
-      <c r="S32" t="s">
+    <row r="28" spans="20:20">
+      <c r="T28" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="33" spans="19:19">
-      <c r="S33" t="s">
+    <row r="29" spans="20:20">
+      <c r="T29" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="34" spans="19:19">
-      <c r="S34" t="s">
+    <row r="30" spans="20:20">
+      <c r="T30" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="35" spans="19:19">
-      <c r="S35" t="s">
+    <row r="31" spans="20:20">
+      <c r="T31" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="36" spans="19:19">
-      <c r="S36" t="s">
+    <row r="32" spans="20:20">
+      <c r="T32" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="37" spans="19:19">
-      <c r="S37" t="s">
+    <row r="33" spans="20:20">
+      <c r="T33" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="38" spans="19:19">
-      <c r="S38" t="s">
+    <row r="34" spans="20:20">
+      <c r="T34" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="39" spans="19:19">
-      <c r="S39" t="s">
+    <row r="35" spans="20:20">
+      <c r="T35" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="40" spans="19:19">
-      <c r="S40" t="s">
+    <row r="36" spans="20:20">
+      <c r="T36" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="41" spans="19:19">
-      <c r="S41" t="s">
+    <row r="37" spans="20:20">
+      <c r="T37" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="42" spans="19:19">
-      <c r="S42" t="s">
+    <row r="38" spans="20:20">
+      <c r="T38" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="43" spans="19:19">
-      <c r="S43" t="s">
+    <row r="39" spans="20:20">
+      <c r="T39" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="44" spans="19:19">
-      <c r="S44" t="s">
+    <row r="40" spans="20:20">
+      <c r="T40" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="45" spans="19:19">
-      <c r="S45" t="s">
+    <row r="41" spans="20:20">
+      <c r="T41" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="46" spans="19:19">
-      <c r="S46" t="s">
+    <row r="42" spans="20:20">
+      <c r="T42" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="47" spans="19:19">
-      <c r="S47" t="s">
+    <row r="43" spans="20:20">
+      <c r="T43" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="48" spans="19:19">
-      <c r="S48" t="s">
+    <row r="44" spans="20:20">
+      <c r="T44" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="49" spans="19:19">
-      <c r="S49" t="s">
+    <row r="45" spans="20:20">
+      <c r="T45" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="50" spans="19:19">
-      <c r="S50" t="s">
+    <row r="46" spans="20:20">
+      <c r="T46" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="51" spans="19:19">
-      <c r="S51" t="s">
+    <row r="47" spans="20:20">
+      <c r="T47" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="52" spans="19:19">
-      <c r="S52" t="s">
+    <row r="48" spans="20:20">
+      <c r="T48" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="53" spans="19:19">
-      <c r="S53" t="s">
+    <row r="49" spans="20:20">
+      <c r="T49" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="54" spans="19:19">
-      <c r="S54" t="s">
+    <row r="50" spans="20:20">
+      <c r="T50" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="55" spans="19:19">
-      <c r="S55" t="s">
+    <row r="51" spans="20:20">
+      <c r="T51" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="56" spans="19:19">
-      <c r="S56" t="s">
+    <row r="52" spans="20:20">
+      <c r="T52" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="57" spans="19:19">
-      <c r="S57" t="s">
+    <row r="53" spans="20:20">
+      <c r="T53" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="58" spans="19:19">
-      <c r="S58" t="s">
+    <row r="54" spans="20:20">
+      <c r="T54" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="59" spans="19:19">
-      <c r="S59" t="s">
+    <row r="55" spans="20:20">
+      <c r="T55" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="60" spans="19:19">
-      <c r="S60" t="s">
+    <row r="56" spans="20:20">
+      <c r="T56" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="61" spans="19:19">
-      <c r="S61" t="s">
+    <row r="57" spans="20:20">
+      <c r="T57" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="62" spans="19:19">
-      <c r="S62" t="s">
+    <row r="58" spans="20:20">
+      <c r="T58" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="63" spans="19:19">
-      <c r="S63" t="s">
+    <row r="59" spans="20:20">
+      <c r="T59" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="64" spans="19:19">
-      <c r="S64" t="s">
+    <row r="60" spans="20:20">
+      <c r="T60" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="65" spans="19:19">
-      <c r="S65" t="s">
+    <row r="61" spans="20:20">
+      <c r="T61" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="66" spans="19:19">
-      <c r="S66" t="s">
+    <row r="62" spans="20:20">
+      <c r="T62" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="67" spans="19:19">
-      <c r="S67" t="s">
+    <row r="63" spans="20:20">
+      <c r="T63" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="68" spans="19:19">
-      <c r="S68" t="s">
+    <row r="64" spans="20:20">
+      <c r="T64" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="69" spans="19:19">
-      <c r="S69" t="s">
+    <row r="65" spans="20:20">
+      <c r="T65" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="70" spans="19:19">
-      <c r="S70" t="s">
+    <row r="66" spans="20:20">
+      <c r="T66" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="71" spans="19:19">
-      <c r="S71" t="s">
+    <row r="67" spans="20:20">
+      <c r="T67" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="72" spans="19:19">
-      <c r="S72" t="s">
+    <row r="68" spans="20:20">
+      <c r="T68" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="73" spans="19:19">
-      <c r="S73" t="s">
+    <row r="69" spans="20:20">
+      <c r="T69" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="74" spans="19:19">
-      <c r="S74" t="s">
+    <row r="70" spans="20:20">
+      <c r="T70" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="75" spans="19:19">
-      <c r="S75" t="s">
+    <row r="71" spans="20:20">
+      <c r="T71" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="76" spans="19:19">
-      <c r="S76" t="s">
+    <row r="72" spans="20:20">
+      <c r="T72" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="77" spans="19:19">
-      <c r="S77" t="s">
+    <row r="73" spans="20:20">
+      <c r="T73" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="78" spans="19:19">
-      <c r="S78" t="s">
+    <row r="74" spans="20:20">
+      <c r="T74" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="79" spans="19:19">
-      <c r="S79" t="s">
+    <row r="75" spans="20:20">
+      <c r="T75" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="80" spans="19:19">
-      <c r="S80" t="s">
+    <row r="76" spans="20:20">
+      <c r="T76" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="81" spans="19:19">
-      <c r="S81" t="s">
+    <row r="77" spans="20:20">
+      <c r="T77" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="82" spans="19:19">
-      <c r="S82" t="s">
+    <row r="78" spans="20:20">
+      <c r="T78" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="83" spans="19:19">
-      <c r="S83" t="s">
+    <row r="79" spans="20:20">
+      <c r="T79" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="84" spans="19:19">
-      <c r="S84" t="s">
+    <row r="80" spans="20:20">
+      <c r="T80" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="85" spans="19:19">
-      <c r="S85" t="s">
+    <row r="81" spans="20:20">
+      <c r="T81" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="86" spans="19:19">
-      <c r="S86" t="s">
+    <row r="82" spans="20:20">
+      <c r="T82" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="87" spans="19:19">
-      <c r="S87" t="s">
+    <row r="83" spans="20:20">
+      <c r="T83" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="88" spans="19:19">
-      <c r="S88" t="s">
+    <row r="84" spans="20:20">
+      <c r="T84" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="89" spans="19:19">
-      <c r="S89" t="s">
+    <row r="85" spans="20:20">
+      <c r="T85" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="90" spans="19:19">
-      <c r="S90" t="s">
+    <row r="86" spans="20:20">
+      <c r="T86" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="91" spans="19:19">
-      <c r="S91" t="s">
+    <row r="87" spans="20:20">
+      <c r="T87" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="92" spans="19:19">
-      <c r="S92" t="s">
+    <row r="88" spans="20:20">
+      <c r="T88" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="93" spans="19:19">
-      <c r="S93" t="s">
+    <row r="89" spans="20:20">
+      <c r="T89" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="94" spans="19:19">
-      <c r="S94" t="s">
+    <row r="90" spans="20:20">
+      <c r="T90" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="95" spans="19:19">
-      <c r="S95" t="s">
+    <row r="91" spans="20:20">
+      <c r="T91" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="96" spans="19:19">
-      <c r="S96" t="s">
+    <row r="92" spans="20:20">
+      <c r="T92" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="97" spans="19:19">
-      <c r="S97" t="s">
+    <row r="93" spans="20:20">
+      <c r="T93" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="98" spans="19:19">
-      <c r="S98" t="s">
+    <row r="94" spans="20:20">
+      <c r="T94" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="99" spans="19:19">
-      <c r="S99" t="s">
+    <row r="95" spans="20:20">
+      <c r="T95" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="100" spans="19:19">
-      <c r="S100" t="s">
+    <row r="96" spans="20:20">
+      <c r="T96" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="101" spans="19:19">
-      <c r="S101" t="s">
+    <row r="97" spans="20:20">
+      <c r="T97" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="102" spans="19:19">
-      <c r="S102" t="s">
+    <row r="98" spans="20:20">
+      <c r="T98" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="103" spans="19:19">
-      <c r="S103" t="s">
+    <row r="99" spans="20:20">
+      <c r="T99" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="104" spans="19:19">
-      <c r="S104" t="s">
+    <row r="100" spans="20:20">
+      <c r="T100" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="105" spans="19:19">
-      <c r="S105" t="s">
+    <row r="101" spans="20:20">
+      <c r="T101" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="106" spans="19:19">
-      <c r="S106" t="s">
+    <row r="102" spans="20:20">
+      <c r="T102" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="107" spans="19:19">
-      <c r="S107" t="s">
+    <row r="103" spans="20:20">
+      <c r="T103" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="108" spans="19:19">
-      <c r="S108" t="s">
+    <row r="104" spans="20:20">
+      <c r="T104" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="109" spans="19:19">
-      <c r="S109" t="s">
+    <row r="105" spans="20:20">
+      <c r="T105" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="110" spans="19:19">
-      <c r="S110" t="s">
+    <row r="106" spans="20:20">
+      <c r="T106" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="111" spans="19:19">
-      <c r="S111" t="s">
+    <row r="107" spans="20:20">
+      <c r="T107" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="112" spans="19:19">
-      <c r="S112" t="s">
+    <row r="108" spans="20:20">
+      <c r="T108" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="113" spans="19:19">
-      <c r="S113" t="s">
+    <row r="109" spans="20:20">
+      <c r="T109" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="114" spans="19:19">
-      <c r="S114" t="s">
+    <row r="110" spans="20:20">
+      <c r="T110" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="115" spans="19:19">
-      <c r="S115" t="s">
+    <row r="111" spans="20:20">
+      <c r="T111" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="116" spans="19:19">
-      <c r="S116" t="s">
+    <row r="112" spans="20:20">
+      <c r="T112" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="117" spans="19:19">
-      <c r="S117" t="s">
+    <row r="113" spans="20:20">
+      <c r="T113" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="118" spans="19:19">
-      <c r="S118" t="s">
+    <row r="114" spans="20:20">
+      <c r="T114" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="119" spans="19:19">
-      <c r="S119" t="s">
+    <row r="115" spans="20:20">
+      <c r="T115" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="120" spans="19:19">
-      <c r="S120" t="s">
+    <row r="116" spans="20:20">
+      <c r="T116" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="121" spans="19:19">
-      <c r="S121" t="s">
+    <row r="117" spans="20:20">
+      <c r="T117" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="122" spans="19:19">
-      <c r="S122" t="s">
+    <row r="118" spans="20:20">
+      <c r="T118" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="123" spans="19:19">
-      <c r="S123" t="s">
+    <row r="119" spans="20:20">
+      <c r="T119" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="124" spans="19:19">
-      <c r="S124" t="s">
+    <row r="120" spans="20:20">
+      <c r="T120" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="125" spans="19:19">
-      <c r="S125" t="s">
+    <row r="121" spans="20:20">
+      <c r="T121" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="126" spans="19:19">
-      <c r="S126" t="s">
+    <row r="122" spans="20:20">
+      <c r="T122" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="127" spans="19:19">
-      <c r="S127" t="s">
+    <row r="123" spans="20:20">
+      <c r="T123" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="128" spans="19:19">
-      <c r="S128" t="s">
+    <row r="124" spans="20:20">
+      <c r="T124" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="129" spans="19:19">
-      <c r="S129" t="s">
+    <row r="125" spans="20:20">
+      <c r="T125" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="130" spans="19:19">
-      <c r="S130" t="s">
+    <row r="126" spans="20:20">
+      <c r="T126" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="131" spans="19:19">
-      <c r="S131" t="s">
+    <row r="127" spans="20:20">
+      <c r="T127" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="132" spans="19:19">
-      <c r="S132" t="s">
+    <row r="128" spans="20:20">
+      <c r="T128" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="133" spans="19:19">
-      <c r="S133" t="s">
+    <row r="129" spans="20:20">
+      <c r="T129" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="134" spans="19:19">
-      <c r="S134" t="s">
+    <row r="130" spans="20:20">
+      <c r="T130" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="135" spans="19:19">
-      <c r="S135" t="s">
+    <row r="131" spans="20:20">
+      <c r="T131" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="136" spans="19:19">
-      <c r="S136" t="s">
+    <row r="132" spans="20:20">
+      <c r="T132" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="137" spans="19:19">
-      <c r="S137" t="s">
+    <row r="133" spans="20:20">
+      <c r="T133" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="138" spans="19:19">
-      <c r="S138" t="s">
+    <row r="134" spans="20:20">
+      <c r="T134" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="139" spans="19:19">
-      <c r="S139" t="s">
+    <row r="135" spans="20:20">
+      <c r="T135" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="140" spans="19:19">
-      <c r="S140" t="s">
+    <row r="136" spans="20:20">
+      <c r="T136" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="141" spans="19:19">
-      <c r="S141" t="s">
+    <row r="137" spans="20:20">
+      <c r="T137" t="s">
         <v>440</v>
       </c>
     </row>
-    <row r="142" spans="19:19">
-      <c r="S142" t="s">
+    <row r="138" spans="20:20">
+      <c r="T138" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="143" spans="19:19">
-      <c r="S143" t="s">
+    <row r="139" spans="20:20">
+      <c r="T139" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="144" spans="19:19">
-      <c r="S144" t="s">
+    <row r="140" spans="20:20">
+      <c r="T140" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="145" spans="19:19">
-      <c r="S145" t="s">
+    <row r="141" spans="20:20">
+      <c r="T141" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="146" spans="19:19">
-      <c r="S146" t="s">
+    <row r="142" spans="20:20">
+      <c r="T142" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="147" spans="19:19">
-      <c r="S147" t="s">
+    <row r="143" spans="20:20">
+      <c r="T143" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="148" spans="19:19">
-      <c r="S148" t="s">
+    <row r="144" spans="20:20">
+      <c r="T144" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="149" spans="19:19">
-      <c r="S149" t="s">
+    <row r="145" spans="20:20">
+      <c r="T145" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="150" spans="19:19">
-      <c r="S150" t="s">
+    <row r="146" spans="20:20">
+      <c r="T146" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="151" spans="19:19">
-      <c r="S151" t="s">
+    <row r="147" spans="20:20">
+      <c r="T147" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="152" spans="19:19">
-      <c r="S152" t="s">
+    <row r="148" spans="20:20">
+      <c r="T148" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="153" spans="19:19">
-      <c r="S153" t="s">
+    <row r="149" spans="20:20">
+      <c r="T149" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="154" spans="19:19">
-      <c r="S154" t="s">
+    <row r="150" spans="20:20">
+      <c r="T150" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="155" spans="19:19">
-      <c r="S155" t="s">
+    <row r="151" spans="20:20">
+      <c r="T151" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="156" spans="19:19">
-      <c r="S156" t="s">
+    <row r="152" spans="20:20">
+      <c r="T152" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="157" spans="19:19">
-      <c r="S157" t="s">
+    <row r="153" spans="20:20">
+      <c r="T153" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="158" spans="19:19">
-      <c r="S158" t="s">
+    <row r="154" spans="20:20">
+      <c r="T154" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="159" spans="19:19">
-      <c r="S159" t="s">
+    <row r="155" spans="20:20">
+      <c r="T155" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="160" spans="19:19">
-      <c r="S160" t="s">
+    <row r="156" spans="20:20">
+      <c r="T156" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="161" spans="19:19">
-      <c r="S161" t="s">
+    <row r="157" spans="20:20">
+      <c r="T157" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="162" spans="19:19">
-      <c r="S162" t="s">
+    <row r="158" spans="20:20">
+      <c r="T158" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="163" spans="19:19">
-      <c r="S163" t="s">
+    <row r="159" spans="20:20">
+      <c r="T159" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="164" spans="19:19">
-      <c r="S164" t="s">
+    <row r="160" spans="20:20">
+      <c r="T160" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="165" spans="19:19">
-      <c r="S165" t="s">
+    <row r="161" spans="20:20">
+      <c r="T161" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="166" spans="19:19">
-      <c r="S166" t="s">
+    <row r="162" spans="20:20">
+      <c r="T162" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="167" spans="19:19">
-      <c r="S167" t="s">
+    <row r="163" spans="20:20">
+      <c r="T163" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="168" spans="19:19">
-      <c r="S168" t="s">
+    <row r="164" spans="20:20">
+      <c r="T164" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="169" spans="19:19">
-      <c r="S169" t="s">
+    <row r="165" spans="20:20">
+      <c r="T165" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="170" spans="19:19">
-      <c r="S170" t="s">
+    <row r="166" spans="20:20">
+      <c r="T166" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="171" spans="19:19">
-      <c r="S171" t="s">
+    <row r="167" spans="20:20">
+      <c r="T167" t="s">
         <v>470</v>
       </c>
     </row>
-    <row r="172" spans="19:19">
-      <c r="S172" t="s">
+    <row r="168" spans="20:20">
+      <c r="T168" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="173" spans="19:19">
-      <c r="S173" t="s">
+    <row r="169" spans="20:20">
+      <c r="T169" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="174" spans="19:19">
-      <c r="S174" t="s">
+    <row r="170" spans="20:20">
+      <c r="T170" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="175" spans="19:19">
-      <c r="S175" t="s">
+    <row r="171" spans="20:20">
+      <c r="T171" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="176" spans="19:19">
-      <c r="S176" t="s">
+    <row r="172" spans="20:20">
+      <c r="T172" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="177" spans="19:19">
-      <c r="S177" t="s">
+    <row r="173" spans="20:20">
+      <c r="T173" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="178" spans="19:19">
-      <c r="S178" t="s">
+    <row r="174" spans="20:20">
+      <c r="T174" t="s">
         <v>477</v>
       </c>
     </row>
-    <row r="179" spans="19:19">
-      <c r="S179" t="s">
+    <row r="175" spans="20:20">
+      <c r="T175" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="180" spans="19:19">
-      <c r="S180" t="s">
+    <row r="176" spans="20:20">
+      <c r="T176" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="181" spans="19:19">
-      <c r="S181" t="s">
+    <row r="177" spans="20:20">
+      <c r="T177" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="182" spans="19:19">
-      <c r="S182" t="s">
+    <row r="178" spans="20:20">
+      <c r="T178" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="183" spans="19:19">
-      <c r="S183" t="s">
+    <row r="179" spans="20:20">
+      <c r="T179" t="s">
         <v>482</v>
       </c>
     </row>
-    <row r="184" spans="19:19">
-      <c r="S184" t="s">
+    <row r="180" spans="20:20">
+      <c r="T180" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="185" spans="19:19">
-      <c r="S185" t="s">
+    <row r="181" spans="20:20">
+      <c r="T181" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="186" spans="19:19">
-      <c r="S186" t="s">
+    <row r="182" spans="20:20">
+      <c r="T182" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="187" spans="19:19">
-      <c r="S187" t="s">
+    <row r="183" spans="20:20">
+      <c r="T183" t="s">
         <v>486</v>
       </c>
     </row>
-    <row r="188" spans="19:19">
-      <c r="S188" t="s">
+    <row r="184" spans="20:20">
+      <c r="T184" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="189" spans="19:19">
-      <c r="S189" t="s">
+    <row r="185" spans="20:20">
+      <c r="T185" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="190" spans="19:19">
-      <c r="S190" t="s">
+    <row r="186" spans="20:20">
+      <c r="T186" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="191" spans="19:19">
-      <c r="S191" t="s">
+    <row r="187" spans="20:20">
+      <c r="T187" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="192" spans="19:19">
-      <c r="S192" t="s">
+    <row r="188" spans="20:20">
+      <c r="T188" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="193" spans="19:19">
-      <c r="S193" t="s">
+    <row r="189" spans="20:20">
+      <c r="T189" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="194" spans="19:19">
-      <c r="S194" t="s">
+    <row r="190" spans="20:20">
+      <c r="T190" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="195" spans="19:19">
-      <c r="S195" t="s">
+    <row r="191" spans="20:20">
+      <c r="T191" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="196" spans="19:19">
-      <c r="S196" t="s">
+    <row r="192" spans="20:20">
+      <c r="T192" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="197" spans="19:19">
-      <c r="S197" t="s">
+    <row r="193" spans="20:20">
+      <c r="T193" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="198" spans="19:19">
-      <c r="S198" t="s">
+    <row r="194" spans="20:20">
+      <c r="T194" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="199" spans="19:19">
-      <c r="S199" t="s">
+    <row r="195" spans="20:20">
+      <c r="T195" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="200" spans="19:19">
-      <c r="S200" t="s">
+    <row r="196" spans="20:20">
+      <c r="T196" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="201" spans="19:19">
-      <c r="S201" t="s">
+    <row r="197" spans="20:20">
+      <c r="T197" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="202" spans="19:19">
-      <c r="S202" t="s">
+    <row r="198" spans="20:20">
+      <c r="T198" t="s">
         <v>501</v>
       </c>
     </row>
-    <row r="203" spans="19:19">
-      <c r="S203" t="s">
+    <row r="199" spans="20:20">
+      <c r="T199" t="s">
         <v>502</v>
       </c>
     </row>
-    <row r="204" spans="19:19">
-      <c r="S204" t="s">
+    <row r="200" spans="20:20">
+      <c r="T200" t="s">
         <v>503</v>
       </c>
     </row>
-    <row r="205" spans="19:19">
-      <c r="S205" t="s">
+    <row r="201" spans="20:20">
+      <c r="T201" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="206" spans="19:19">
-      <c r="S206" t="s">
+    <row r="202" spans="20:20">
+      <c r="T202" t="s">
         <v>505</v>
       </c>
     </row>
-    <row r="207" spans="19:19">
-      <c r="S207" t="s">
+    <row r="203" spans="20:20">
+      <c r="T203" t="s">
         <v>506</v>
       </c>
     </row>
-    <row r="208" spans="19:19">
-      <c r="S208" t="s">
+    <row r="204" spans="20:20">
+      <c r="T204" t="s">
         <v>507</v>
       </c>
     </row>
-    <row r="209" spans="19:19">
-      <c r="S209" t="s">
+    <row r="205" spans="20:20">
+      <c r="T205" t="s">
         <v>508</v>
       </c>
     </row>
-    <row r="210" spans="19:19">
-      <c r="S210" t="s">
+    <row r="206" spans="20:20">
+      <c r="T206" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="211" spans="19:19">
-      <c r="S211" t="s">
+    <row r="207" spans="20:20">
+      <c r="T207" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="212" spans="19:19">
-      <c r="S212" t="s">
+    <row r="208" spans="20:20">
+      <c r="T208" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="213" spans="19:19">
-      <c r="S213" t="s">
+    <row r="209" spans="20:20">
+      <c r="T209" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="214" spans="19:19">
-      <c r="S214" t="s">
+    <row r="210" spans="20:20">
+      <c r="T210" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="215" spans="19:19">
-      <c r="S215" t="s">
+    <row r="211" spans="20:20">
+      <c r="T211" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="216" spans="19:19">
-      <c r="S216" t="s">
+    <row r="212" spans="20:20">
+      <c r="T212" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="217" spans="19:19">
-      <c r="S217" t="s">
+    <row r="213" spans="20:20">
+      <c r="T213" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="218" spans="19:19">
-      <c r="S218" t="s">
+    <row r="214" spans="20:20">
+      <c r="T214" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="219" spans="19:19">
-      <c r="S219" t="s">
+    <row r="215" spans="20:20">
+      <c r="T215" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="220" spans="19:19">
-      <c r="S220" t="s">
+    <row r="216" spans="20:20">
+      <c r="T216" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="221" spans="19:19">
-      <c r="S221" t="s">
+    <row r="217" spans="20:20">
+      <c r="T217" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="222" spans="19:19">
-      <c r="S222" t="s">
+    <row r="218" spans="20:20">
+      <c r="T218" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="223" spans="19:19">
-      <c r="S223" t="s">
+    <row r="219" spans="20:20">
+      <c r="T219" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="224" spans="19:19">
-      <c r="S224" t="s">
+    <row r="220" spans="20:20">
+      <c r="T220" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="225" spans="19:19">
-      <c r="S225" t="s">
+    <row r="221" spans="20:20">
+      <c r="T221" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="226" spans="19:19">
-      <c r="S226" t="s">
+    <row r="222" spans="20:20">
+      <c r="T222" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="227" spans="19:19">
-      <c r="S227" t="s">
+    <row r="223" spans="20:20">
+      <c r="T223" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="228" spans="19:19">
-      <c r="S228" t="s">
+    <row r="224" spans="20:20">
+      <c r="T224" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="229" spans="19:19">
-      <c r="S229" t="s">
+    <row r="225" spans="20:20">
+      <c r="T225" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="230" spans="19:19">
-      <c r="S230" t="s">
+    <row r="226" spans="20:20">
+      <c r="T226" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="231" spans="19:19">
-      <c r="S231" t="s">
+    <row r="227" spans="20:20">
+      <c r="T227" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="232" spans="19:19">
-      <c r="S232" t="s">
+    <row r="228" spans="20:20">
+      <c r="T228" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="233" spans="19:19">
-      <c r="S233" t="s">
+    <row r="229" spans="20:20">
+      <c r="T229" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="234" spans="19:19">
-      <c r="S234" t="s">
+    <row r="230" spans="20:20">
+      <c r="T230" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="235" spans="19:19">
-      <c r="S235" t="s">
+    <row r="231" spans="20:20">
+      <c r="T231" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="236" spans="19:19">
-      <c r="S236" t="s">
+    <row r="232" spans="20:20">
+      <c r="T232" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="237" spans="19:19">
-      <c r="S237" t="s">
+    <row r="233" spans="20:20">
+      <c r="T233" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="238" spans="19:19">
-      <c r="S238" t="s">
+    <row r="234" spans="20:20">
+      <c r="T234" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="239" spans="19:19">
-      <c r="S239" t="s">
+    <row r="235" spans="20:20">
+      <c r="T235" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="240" spans="19:19">
-      <c r="S240" t="s">
+    <row r="236" spans="20:20">
+      <c r="T236" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="241" spans="19:19">
-      <c r="S241" t="s">
+    <row r="237" spans="20:20">
+      <c r="T237" t="s">
         <v>540</v>
       </c>
     </row>
-    <row r="242" spans="19:19">
-      <c r="S242" t="s">
+    <row r="238" spans="20:20">
+      <c r="T238" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="243" spans="19:19">
-      <c r="S243" t="s">
+    <row r="239" spans="20:20">
+      <c r="T239" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="244" spans="19:19">
-      <c r="S244" t="s">
+    <row r="240" spans="20:20">
+      <c r="T240" t="s">
         <v>543</v>
       </c>
     </row>
-    <row r="245" spans="19:19">
-      <c r="S245" t="s">
+    <row r="241" spans="20:20">
+      <c r="T241" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="246" spans="19:19">
-      <c r="S246" t="s">
+    <row r="242" spans="20:20">
+      <c r="T242" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="247" spans="19:19">
-      <c r="S247" t="s">
+    <row r="243" spans="20:20">
+      <c r="T243" t="s">
         <v>546</v>
       </c>
     </row>
-    <row r="248" spans="19:19">
-      <c r="S248" t="s">
+    <row r="244" spans="20:20">
+      <c r="T244" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="249" spans="19:19">
-      <c r="S249" t="s">
+    <row r="245" spans="20:20">
+      <c r="T245" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="250" spans="19:19">
-      <c r="S250" t="s">
+    <row r="246" spans="20:20">
+      <c r="T246" t="s">
         <v>549</v>
       </c>
     </row>
-    <row r="251" spans="19:19">
-      <c r="S251" t="s">
+    <row r="247" spans="20:20">
+      <c r="T247" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="252" spans="19:19">
-      <c r="S252" t="s">
+    <row r="248" spans="20:20">
+      <c r="T248" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="253" spans="19:19">
-      <c r="S253" t="s">
+    <row r="249" spans="20:20">
+      <c r="T249" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="254" spans="19:19">
-      <c r="S254" t="s">
+    <row r="250" spans="20:20">
+      <c r="T250" t="s">
         <v>553</v>
       </c>
     </row>
-    <row r="255" spans="19:19">
-      <c r="S255" t="s">
+    <row r="251" spans="20:20">
+      <c r="T251" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="256" spans="19:19">
-      <c r="S256" t="s">
+    <row r="252" spans="20:20">
+      <c r="T252" t="s">
         <v>555</v>
       </c>
     </row>
-    <row r="257" spans="19:19">
-      <c r="S257" t="s">
+    <row r="253" spans="20:20">
+      <c r="T253" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="258" spans="19:19">
-      <c r="S258" t="s">
+    <row r="254" spans="20:20">
+      <c r="T254" t="s">
         <v>557</v>
       </c>
     </row>
-    <row r="259" spans="19:19">
-      <c r="S259" t="s">
+    <row r="255" spans="20:20">
+      <c r="T255" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="260" spans="19:19">
-      <c r="S260" t="s">
+    <row r="256" spans="20:20">
+      <c r="T256" t="s">
         <v>559</v>
       </c>
     </row>
-    <row r="261" spans="19:19">
-      <c r="S261" t="s">
+    <row r="257" spans="20:20">
+      <c r="T257" t="s">
         <v>560</v>
       </c>
     </row>
-    <row r="262" spans="19:19">
-      <c r="S262" t="s">
+    <row r="258" spans="20:20">
+      <c r="T258" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="263" spans="19:19">
-      <c r="S263" t="s">
+    <row r="259" spans="20:20">
+      <c r="T259" t="s">
         <v>562</v>
       </c>
     </row>
-    <row r="264" spans="19:19">
-      <c r="S264" t="s">
+    <row r="260" spans="20:20">
+      <c r="T260" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="265" spans="19:19">
-      <c r="S265" t="s">
+    <row r="261" spans="20:20">
+      <c r="T261" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="266" spans="19:19">
-      <c r="S266" t="s">
+    <row r="262" spans="20:20">
+      <c r="T262" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="267" spans="19:19">
-      <c r="S267" t="s">
+    <row r="263" spans="20:20">
+      <c r="T263" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="268" spans="19:19">
-      <c r="S268" t="s">
+    <row r="264" spans="20:20">
+      <c r="T264" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="269" spans="19:19">
-      <c r="S269" t="s">
+    <row r="265" spans="20:20">
+      <c r="T265" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="270" spans="19:19">
-      <c r="S270" t="s">
+    <row r="266" spans="20:20">
+      <c r="T266" t="s">
         <v>569</v>
       </c>
     </row>
-    <row r="271" spans="19:19">
-      <c r="S271" t="s">
+    <row r="267" spans="20:20">
+      <c r="T267" t="s">
         <v>570</v>
       </c>
     </row>
-    <row r="272" spans="19:19">
-      <c r="S272" t="s">
+    <row r="268" spans="20:20">
+      <c r="T268" t="s">
         <v>571</v>
       </c>
     </row>
-    <row r="273" spans="19:19">
-      <c r="S273" t="s">
+    <row r="269" spans="20:20">
+      <c r="T269" t="s">
         <v>572</v>
       </c>
     </row>
-    <row r="274" spans="19:19">
-      <c r="S274" t="s">
+    <row r="270" spans="20:20">
+      <c r="T270" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="275" spans="19:19">
-      <c r="S275" t="s">
+    <row r="271" spans="20:20">
+      <c r="T271" t="s">
         <v>574</v>
       </c>
     </row>
-    <row r="276" spans="19:19">
-      <c r="S276" t="s">
+    <row r="272" spans="20:20">
+      <c r="T272" t="s">
         <v>575</v>
       </c>
     </row>
-    <row r="277" spans="19:19">
-      <c r="S277" t="s">
+    <row r="273" spans="20:20">
+      <c r="T273" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="278" spans="19:19">
-      <c r="S278" t="s">
+    <row r="274" spans="20:20">
+      <c r="T274" t="s">
         <v>577</v>
       </c>
     </row>
-    <row r="279" spans="19:19">
-      <c r="S279" t="s">
+    <row r="275" spans="20:20">
+      <c r="T275" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="280" spans="19:19">
-      <c r="S280" t="s">
+    <row r="276" spans="20:20">
+      <c r="T276" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="281" spans="19:19">
-      <c r="S281" t="s">
+    <row r="277" spans="20:20">
+      <c r="T277" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="282" spans="19:19">
-      <c r="S282" t="s">
+    <row r="278" spans="20:20">
+      <c r="T278" t="s">
         <v>581</v>
       </c>
     </row>
-    <row r="283" spans="19:19">
-      <c r="S283" t="s">
+    <row r="279" spans="20:20">
+      <c r="T279" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="284" spans="19:19">
-      <c r="S284" t="s">
+    <row r="280" spans="20:20">
+      <c r="T280" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="285" spans="19:19">
-      <c r="S285" t="s">
+    <row r="281" spans="20:20">
+      <c r="T281" t="s">
         <v>584</v>
       </c>
     </row>
-    <row r="286" spans="19:19">
-      <c r="S286" t="s">
+    <row r="282" spans="20:20">
+      <c r="T282" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="287" spans="19:19">
-      <c r="S287" t="s">
+    <row r="283" spans="20:20">
+      <c r="T283" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="288" spans="19:19">
-      <c r="S288" t="s">
+    <row r="284" spans="20:20">
+      <c r="T284" t="s">
         <v>587</v>
       </c>
     </row>
-    <row r="289" spans="19:19">
-      <c r="S289" t="s">
+    <row r="285" spans="20:20">
+      <c r="T285" t="s">
         <v>588</v>
+      </c>
+    </row>
+    <row r="286" spans="20:20">
+      <c r="T286" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="287" spans="20:20">
+      <c r="T287" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="288" spans="20:20">
+      <c r="T288" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="289" spans="20:20">
+      <c r="T289" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="290" spans="20:20">
+      <c r="T290" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="291" spans="20:20">
+      <c r="T291" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="292" spans="20:20">
+      <c r="T292" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="293" spans="20:20">
+      <c r="T293" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="294" spans="20:20">
+      <c r="T294" t="s">
+        <v>597</v>
       </c>
     </row>
   </sheetData>

</xml_diff>